<commit_message>
Fixes due to website upadates
</commit_message>
<xml_diff>
--- a/top_250_data.xlsx
+++ b/top_250_data.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,26 +413,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D323"/>
+  <dimension ref="A1:D371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>tmdbID</t>
         </is>
@@ -6388,10 +6376,8 @@
           <t>BTS WORLD TOUR [LOVE YOURSELF : SPEAK YOURSELF] in London Remastered</t>
         </is>
       </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+      <c r="B320" t="n">
+        <v>2025</v>
       </c>
       <c r="C320" t="inlineStr">
         <is>
@@ -6410,10 +6396,8 @@
           <t>BTS WORLD TOUR [ARIRANG] in Goyang</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
+      <c r="B321" t="n">
+        <v>2026</v>
       </c>
       <c r="C321" t="inlineStr">
         <is>
@@ -6432,10 +6416,8 @@
           <t>BTS: Permission to Dance on Stage - Seoul</t>
         </is>
       </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
+      <c r="B322" t="n">
+        <v>2022</v>
       </c>
       <c r="C322" t="inlineStr">
         <is>
@@ -6454,10 +6436,8 @@
           <t>War and Peace</t>
         </is>
       </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>1967</t>
-        </is>
+      <c r="B323" t="n">
+        <v>1967</v>
       </c>
       <c r="C323" t="inlineStr">
         <is>
@@ -6467,6 +6447,954 @@
       <c r="D323" t="inlineStr">
         <is>
           <t>29266</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>My Dearest</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/my-dearest-2023/</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>SUGA | Agust D TOUR [D-DAY] in Japan</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/suga-agust-d-tour-d-day-in-japan/</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>1124669</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>5 Seconds of Summer: The Feeling of Falling Upwards - Live from Royal Albert Hall</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/5-seconds-of-summer-the-feeling-of-falling-upwards-live-from-royal-albert-hall/</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>1018688</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Cyberpunk: Edgerunners</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/cyberpunk-edgerunners/</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Good Will Hunting</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>1997</v>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/good-will-hunting/</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>489</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>BTS WORLD TOUR [ARIRANG] in Japan</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/bts-world-tour-arirang-in-japan/</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>1640677</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Orb: On the Movements of the Earth</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/orb-on-the-movements-of-the-earth/</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Ditto</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/ditto-2022-1/</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>1614301</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Se7en</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>1995</v>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/se7en/</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>807</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>An Elephant Sitting Still</t>
+        </is>
+      </c>
+      <c r="B333" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/an-elephant-sitting-still/</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>499556</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>It's Always Sunny In Philadelphia: Sunny Side Up</t>
+        </is>
+      </c>
+      <c r="B334" t="n">
+        <v>2007</v>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/its-always-sunny-in-philadelphia-sunny-side-up/</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>1060033</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>RM: Right People, Wrong Place</t>
+        </is>
+      </c>
+      <c r="B335" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/rm-right-people-wrong-place/</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>1346709</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Black Country, New Road - “Live at Bush Hall”</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/black-country-new-road-live-at-bush-hall/</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>1139769</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>SEVENTEEN TOUR 'FOLLOW' AGAIN TO CINEMAS</t>
+        </is>
+      </c>
+      <c r="B337" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/seventeen-tour-follow-again-to-cinemas/</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>1317874</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Hans Zimmer: Live in Prague</t>
+        </is>
+      </c>
+      <c r="B338" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/hans-zimmer-live-in-prague/</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>435011</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>The Apothecary Diaries</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/the-apothecary-diaries/</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Gurren Lagann</t>
+        </is>
+      </c>
+      <c r="B340" t="n">
+        <v>2007</v>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/gurren-lagann/</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Linkin Park: Live in Texas</t>
+        </is>
+      </c>
+      <c r="B341" t="n">
+        <v>2003</v>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/linkin-park-live-in-texas/</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>40444</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="B342" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/mouse-2021-1/</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="B343" t="n">
+        <v>1969</v>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/z/</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>2721</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Lemonade</t>
+        </is>
+      </c>
+      <c r="B344" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/lemonade-2016/</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>394269</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Apur Sansar</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>1959</v>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/apur-sansar/</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>896</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Harlan County U.S.A.</t>
+        </is>
+      </c>
+      <c r="B346" t="n">
+        <v>1976</v>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/harlan-county-usa/</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>33324</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Code Geass: Lelouch of the Rebellion R2 Special Edition - Zero Requiem</t>
+        </is>
+      </c>
+      <c r="B347" t="n">
+        <v>2009</v>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/code-geass-lelouch-of-the-rebellion-r2-special-edition-zero-requiem/</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>1263462</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Lucky Three: An Elliott Smith Portrait</t>
+        </is>
+      </c>
+      <c r="B348" t="n">
+        <v>1997</v>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/lucky-three-an-elliott-smith-portrait/</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>144501</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>One Direction: Where We Are - The Concert Film</t>
+        </is>
+      </c>
+      <c r="B349" t="n">
+        <v>2014</v>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/one-direction-where-we-are-the-concert-film/</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>283559</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>BTS Monuments: Beyond the Star</t>
+        </is>
+      </c>
+      <c r="B350" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/bts-monuments-beyond-the-star-2023/</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>CALL ME IF YOU GET LOST LIVE</t>
+        </is>
+      </c>
+      <c r="B351" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/call-me-if-you-get-lost-live/</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>956007</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Moving</t>
+        </is>
+      </c>
+      <c r="B352" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/moving-2023-1/</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>One Flew Over the Cuckoo's Nest</t>
+        </is>
+      </c>
+      <c r="B353" t="n">
+        <v>1975</v>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/one-flew-over-the-cuckoos-nest/</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>510</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Apple Music Live: Gracie Abrams</t>
+        </is>
+      </c>
+      <c r="B354" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/apple-music-live-gracie-abrams/</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>1565821</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Radiohead: The King of Limbs – Live from the Basement</t>
+        </is>
+      </c>
+      <c r="B355" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/radiohead-the-king-of-limbs-live-from-the/</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>152940</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>How to Make Millions Before Grandma Dies</t>
+        </is>
+      </c>
+      <c r="B356" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/how-to-make-millions-before-grandma-dies/</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>1103621</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Judgment at Nuremberg</t>
+        </is>
+      </c>
+      <c r="B357" t="n">
+        <v>1961</v>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/judgment-at-nuremberg/</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>821</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Amadeus</t>
+        </is>
+      </c>
+      <c r="B358" t="n">
+        <v>1984</v>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/amadeus/</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>279</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Inglourious Basterds</t>
+        </is>
+      </c>
+      <c r="B359" t="n">
+        <v>2009</v>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/inglourious-basterds/</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>16869</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>BTS Live Trilogy Episode III: The Wings Tour in Seoul</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/bts-live-trilogy-episode-iii-the-wings-tour-2025/</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>1538059</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Ikebukuro West Gate Park</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/ikebukuro-west-gate-park/</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Billie Eilish: Live at the O2</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/billie-eilish-live-at-the-o2-extended-cut/</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>1058923</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>20 Days in Mariupol</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/20-days-in-mariupol/</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>1058616</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>A Modern Farewell</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/a-modern-farewell/</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>699283</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>It's Never Over, Jeff Buckley</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/its-never-over-jeff-buckley/</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>1400381</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>The Beaches of Agnès</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/the-beaches-of-agnes/</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>38879</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Pride and Prejudice</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/pride-and-prejudice-1995/</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>452736</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Heat</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/heat-1995/</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Brighter Days Ahead</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/brighter-days-ahead/</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>1447182</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Late Spring</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>1949</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/late-spring/</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>20530</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>BTS WORLD TOUR [LOVE YOURSELF] in Seoul</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/bts-world-tour-love-yourself-in-seoul/</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>568300</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixes for chrome time outs
</commit_message>
<xml_diff>
--- a/top_250_data.xlsx
+++ b/top_250_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D407"/>
+  <dimension ref="A1:D408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8064,10 +8064,8 @@
           <t>Daft Punk: Alive 2007 - Live Album Concert in Paris</t>
         </is>
       </c>
-      <c r="B407" t="inlineStr">
-        <is>
-          <t>2007</t>
-        </is>
+      <c r="B407" t="n">
+        <v>2007</v>
       </c>
       <c r="C407" t="inlineStr">
         <is>
@@ -8077,6 +8075,28 @@
       <c r="D407" t="inlineStr">
         <is>
           <t>843809</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>NAZA</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/naza/</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>1755291</t>
         </is>
       </c>
     </row>

</xml_diff>